<commit_message>
Renamed main files to avoid confusion
</commit_message>
<xml_diff>
--- a/Pressurization_System/Press System Test Cases.xlsx
+++ b/Pressurization_System/Press System Test Cases.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brigh\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://purdue0-my.sharepoint.com/personal/tucke193_purdue_edu/Documents/PSP/Test Stand/PSPL_Test_Stand/Pressurization_System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3BA32EE1-FD8D-41E0-A269-E64256623536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="8_{3BA32EE1-FD8D-41E0-A269-E64256623536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5648216-8155-4EF9-ACC8-404ED47825BC}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C0027B85-AECA-41BE-812F-CA93B39DA64E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{C0027B85-AECA-41BE-812F-CA93B39DA64E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Initial Conditions" sheetId="1" r:id="rId1"/>
+    <sheet name="Configurations" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
   <si>
     <t>Oxidizer</t>
   </si>
@@ -50,28 +51,61 @@
     <t>Fu Press Gas</t>
   </si>
   <si>
-    <t>OX mdot</t>
-  </si>
-  <si>
-    <t>FU mdot</t>
-  </si>
-  <si>
-    <t>Source Pressure</t>
-  </si>
-  <si>
-    <t>Source Temperature</t>
-  </si>
-  <si>
-    <t>Fill Pressure (used for prop density)</t>
-  </si>
-  <si>
     <t>Single/Dual Source</t>
   </si>
   <si>
-    <t>Tank Pressure</t>
-  </si>
-  <si>
     <t>Test Case Description</t>
+  </si>
+  <si>
+    <t>OX mdot (kg/s)</t>
+  </si>
+  <si>
+    <t>FU mdot (kg/s)</t>
+  </si>
+  <si>
+    <t>Tank Pressure (psi)</t>
+  </si>
+  <si>
+    <t>Fill Pressure (used for prop density) (psi)</t>
+  </si>
+  <si>
+    <t>Ox Source Pressure (psi)</t>
+  </si>
+  <si>
+    <t>Ox Source Temperature (K)</t>
+  </si>
+  <si>
+    <t>Fu Source Pressure (psi)</t>
+  </si>
+  <si>
+    <t>Fu Source Temperature (K)</t>
+  </si>
+  <si>
+    <t>5000lbf Main Test</t>
+  </si>
+  <si>
+    <t>LOX</t>
+  </si>
+  <si>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Valve</t>
+  </si>
+  <si>
+    <t>Tube</t>
+  </si>
+  <si>
+    <t>Regulator</t>
+  </si>
+  <si>
+    <t>Length (ft)</t>
+  </si>
+  <si>
+    <t>Diameter (in)</t>
+  </si>
+  <si>
+    <t>Cv (dimensionless)</t>
   </si>
 </sst>
 </file>
@@ -124,6 +158,42 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6035B4D9-1642-4FDC-83F9-A202C56D97BF}" name="Table1" displayName="Table1" ref="A1:N3" totalsRowShown="0">
+  <autoFilter ref="A1:N3" xr:uid="{6035B4D9-1642-4FDC-83F9-A202C56D97BF}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{F1F2B89A-0182-47BD-AF47-28EBC8F67DC5}" name="Test Case Description"/>
+    <tableColumn id="2" xr3:uid="{028B1448-36D6-4C7B-83A2-D697C29BD4E1}" name="Oxidizer"/>
+    <tableColumn id="3" xr3:uid="{AC0C8ABE-2138-46AF-838C-CE23E35B4A09}" name="OX mdot (kg/s)"/>
+    <tableColumn id="4" xr3:uid="{1C2FF809-5FFB-459A-B5D7-42BEF4C04AA2}" name="FU mdot (kg/s)"/>
+    <tableColumn id="5" xr3:uid="{6F1CAFC6-53BA-4008-ABF6-539843B7C312}" name="Fuel"/>
+    <tableColumn id="6" xr3:uid="{26ED1644-701B-48D2-988A-F7E06B9F8F47}" name="Single/Dual Source"/>
+    <tableColumn id="7" xr3:uid="{A89FC2E7-A5A5-4B36-A697-D725530FD1AF}" name="Tank Pressure (psi)"/>
+    <tableColumn id="8" xr3:uid="{7659E010-E8AA-4FAC-86E8-2222973BDFFE}" name="Fill Pressure (used for prop density) (psi)"/>
+    <tableColumn id="9" xr3:uid="{A64DC4F4-A184-4D0B-8E07-BC4209542B83}" name="Ox Press Gas"/>
+    <tableColumn id="10" xr3:uid="{3F2BA43E-8364-4D07-8B5F-8A76FB3F8E6E}" name="Ox Source Pressure (psi)"/>
+    <tableColumn id="11" xr3:uid="{375A1EBD-2658-41BB-A916-BF3F722D5A95}" name="Ox Source Temperature (K)"/>
+    <tableColumn id="12" xr3:uid="{516A76CC-8D45-4E24-9F7F-142004617BC1}" name="Fu Press Gas"/>
+    <tableColumn id="13" xr3:uid="{5BB4A00F-DA34-4B22-A583-3BCE9D881BFE}" name="Fu Source Pressure (psi)"/>
+    <tableColumn id="14" xr3:uid="{303A5C50-F899-4E2C-B94B-A2D11BB69A68}" name="Fu Source Temperature (K)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3398EC84-E190-48C4-9758-828E3B516797}" name="Table3" displayName="Table3" ref="A1:D8" totalsRowShown="0">
+  <autoFilter ref="A1:D8" xr:uid="{3398EC84-E190-48C4-9758-828E3B516797}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{E1C86204-DEAE-4724-8EA6-A47D0CD8B514}" name="Component"/>
+    <tableColumn id="2" xr3:uid="{B219FCE6-DF04-4AB9-84BB-9F16F91F6C3A}" name="Length (ft)"/>
+    <tableColumn id="3" xr3:uid="{993BB252-BCF7-4652-8EB4-BE888A84B7EA}" name="Diameter (in)"/>
+    <tableColumn id="4" xr3:uid="{AFD5FEAB-FF1F-4E72-AA07-4AD4714427A1}" name="Cv (dimensionless)"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -443,74 +513,149 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7708522A-A771-4A2F-B747-04EC8410C62A}">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="32.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="41" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" t="s">
+      <c r="I1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>10</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" t="s">
-        <v>7</v>
-      </c>
-      <c r="L1" t="s">
-        <v>10</v>
-      </c>
       <c r="M1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>5</v>
-      </c>
-      <c r="O1" t="s">
-        <v>8</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{088C9C01-56F8-4798-8850-4C6BA490C79B}">
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Lots more calculations done (PRE-PDR)
</commit_message>
<xml_diff>
--- a/Pressurization_System/Press System Test Cases.xlsx
+++ b/Pressurization_System/Press System Test Cases.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://purdue0-my.sharepoint.com/personal/tucke193_purdue_edu/Documents/PSP/Test Stand/PSPL_Test_Stand/Pressurization_System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="65" documentId="8_{3BA32EE1-FD8D-41E0-A269-E64256623536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5648216-8155-4EF9-ACC8-404ED47825BC}"/>
+  <xr:revisionPtr revIDLastSave="349" documentId="8_{3BA32EE1-FD8D-41E0-A269-E64256623536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F25E5AB-9888-4037-ACA2-3C0026F22B04}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{C0027B85-AECA-41BE-812F-CA93B39DA64E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C0027B85-AECA-41BE-812F-CA93B39DA64E}"/>
   </bookViews>
   <sheets>
     <sheet name="Initial Conditions" sheetId="1" r:id="rId1"/>
-    <sheet name="Configurations" sheetId="2" r:id="rId2"/>
+    <sheet name="Configuration 1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>Oxidizer</t>
   </si>
@@ -45,12 +45,6 @@
     <t>Fuel</t>
   </si>
   <si>
-    <t>Ox Press Gas</t>
-  </si>
-  <si>
-    <t>Fu Press Gas</t>
-  </si>
-  <si>
     <t>Single/Dual Source</t>
   </si>
   <si>
@@ -63,56 +57,92 @@
     <t>FU mdot (kg/s)</t>
   </si>
   <si>
-    <t>Tank Pressure (psi)</t>
-  </si>
-  <si>
     <t>Fill Pressure (used for prop density) (psi)</t>
   </si>
   <si>
-    <t>Ox Source Pressure (psi)</t>
-  </si>
-  <si>
-    <t>Ox Source Temperature (K)</t>
-  </si>
-  <si>
-    <t>Fu Source Pressure (psi)</t>
-  </si>
-  <si>
-    <t>Fu Source Temperature (K)</t>
-  </si>
-  <si>
-    <t>5000lbf Main Test</t>
+    <t>Component</t>
+  </si>
+  <si>
+    <t>Valve</t>
+  </si>
+  <si>
+    <t>Tube</t>
+  </si>
+  <si>
+    <t>Regulator</t>
+  </si>
+  <si>
+    <t>Length (ft)</t>
+  </si>
+  <si>
+    <t>Diameter (in)</t>
+  </si>
+  <si>
+    <t>Cv (dimensionless)</t>
+  </si>
+  <si>
+    <t>OX Tank Pressure (psi)</t>
+  </si>
+  <si>
+    <t>Tank Volume (ft^3)</t>
+  </si>
+  <si>
+    <t>FU Tank Pressure (psi)</t>
+  </si>
+  <si>
+    <t>OX Press Gas</t>
+  </si>
+  <si>
+    <t>OX Source Pressure (psi)</t>
+  </si>
+  <si>
+    <t>OX Source Temperature (K)</t>
+  </si>
+  <si>
+    <t>FU Press Gas</t>
+  </si>
+  <si>
+    <t>FU Source Pressure (psi)</t>
+  </si>
+  <si>
+    <t>FU Source Temperature (K)</t>
+  </si>
+  <si>
+    <t>Configuration No.</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>Oxygen</t>
+  </si>
+  <si>
+    <t>Test Case Number</t>
+  </si>
+  <si>
+    <t>Combined</t>
   </si>
   <si>
     <t>LOX</t>
   </si>
   <si>
-    <t>Component</t>
-  </si>
-  <si>
-    <t>Valve</t>
-  </si>
-  <si>
-    <t>Tube</t>
-  </si>
-  <si>
-    <t>Regulator</t>
-  </si>
-  <si>
-    <t>Length (ft)</t>
-  </si>
-  <si>
-    <t>Diameter (in)</t>
-  </si>
-  <si>
-    <t>Cv (dimensionless)</t>
+    <t>Fu</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>Ethanol</t>
+  </si>
+  <si>
+    <t>Primary</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,16 +150,61 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -137,17 +212,78 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -160,37 +296,36 @@
 </styleSheet>
 </file>
 
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6035B4D9-1642-4FDC-83F9-A202C56D97BF}" name="Table1" displayName="Table1" ref="A1:N3" totalsRowShown="0">
-  <autoFilter ref="A1:N3" xr:uid="{6035B4D9-1642-4FDC-83F9-A202C56D97BF}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{F1F2B89A-0182-47BD-AF47-28EBC8F67DC5}" name="Test Case Description"/>
-    <tableColumn id="2" xr3:uid="{028B1448-36D6-4C7B-83A2-D697C29BD4E1}" name="Oxidizer"/>
-    <tableColumn id="3" xr3:uid="{AC0C8ABE-2138-46AF-838C-CE23E35B4A09}" name="OX mdot (kg/s)"/>
-    <tableColumn id="4" xr3:uid="{1C2FF809-5FFB-459A-B5D7-42BEF4C04AA2}" name="FU mdot (kg/s)"/>
-    <tableColumn id="5" xr3:uid="{6F1CAFC6-53BA-4008-ABF6-539843B7C312}" name="Fuel"/>
-    <tableColumn id="6" xr3:uid="{26ED1644-701B-48D2-988A-F7E06B9F8F47}" name="Single/Dual Source"/>
-    <tableColumn id="7" xr3:uid="{A89FC2E7-A5A5-4B36-A697-D725530FD1AF}" name="Tank Pressure (psi)"/>
-    <tableColumn id="8" xr3:uid="{7659E010-E8AA-4FAC-86E8-2222973BDFFE}" name="Fill Pressure (used for prop density) (psi)"/>
-    <tableColumn id="9" xr3:uid="{A64DC4F4-A184-4D0B-8E07-BC4209542B83}" name="Ox Press Gas"/>
-    <tableColumn id="10" xr3:uid="{3F2BA43E-8364-4D07-8B5F-8A76FB3F8E6E}" name="Ox Source Pressure (psi)"/>
-    <tableColumn id="11" xr3:uid="{375A1EBD-2658-41BB-A916-BF3F722D5A95}" name="Ox Source Temperature (K)"/>
-    <tableColumn id="12" xr3:uid="{516A76CC-8D45-4E24-9F7F-142004617BC1}" name="Fu Press Gas"/>
-    <tableColumn id="13" xr3:uid="{5BB4A00F-DA34-4B22-A583-3BCE9D881BFE}" name="Fu Source Pressure (psi)"/>
-    <tableColumn id="14" xr3:uid="{303A5C50-F899-4E2C-B94B-A2D11BB69A68}" name="Fu Source Temperature (K)"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{3398EC84-E190-48C4-9758-828E3B516797}" name="Table3" displayName="Table3" ref="A1:D8" totalsRowShown="0">
-  <autoFilter ref="A1:D8" xr:uid="{3398EC84-E190-48C4-9758-828E3B516797}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{E1C86204-DEAE-4724-8EA6-A47D0CD8B514}" name="Component"/>
-    <tableColumn id="2" xr3:uid="{B219FCE6-DF04-4AB9-84BB-9F16F91F6C3A}" name="Length (ft)"/>
-    <tableColumn id="3" xr3:uid="{993BB252-BCF7-4652-8EB4-BE888A84B7EA}" name="Diameter (in)"/>
-    <tableColumn id="4" xr3:uid="{AFD5FEAB-FF1F-4E72-AA07-4AD4714427A1}" name="Cv (dimensionless)"/>
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6035B4D9-1642-4FDC-83F9-A202C56D97BF}" name="Table1" displayName="Table1" ref="A1:R2" totalsRowShown="0">
+  <autoFilter ref="A1:R2" xr:uid="{6035B4D9-1642-4FDC-83F9-A202C56D97BF}"/>
+  <tableColumns count="18">
+    <tableColumn id="18" xr3:uid="{01F791EE-3033-4427-BCC2-BA393292DEED}" name="Test Case Number"/>
+    <tableColumn id="1" xr3:uid="{F1F2B89A-0182-47BD-AF47-28EBC8F67DC5}" name="Test Case Description"/>
+    <tableColumn id="17" xr3:uid="{769BF319-34C2-4202-9D5A-FD7182836356}" name="Configuration No."/>
+    <tableColumn id="6" xr3:uid="{26ED1644-701B-48D2-988A-F7E06B9F8F47}" name="Single/Dual Source"/>
+    <tableColumn id="15" xr3:uid="{4291074D-C4DD-4453-B948-5D9BEC6801CE}" name="Tank Volume (ft^3)"/>
+    <tableColumn id="2" xr3:uid="{028B1448-36D6-4C7B-83A2-D697C29BD4E1}" name="Oxidizer"/>
+    <tableColumn id="3" xr3:uid="{AC0C8ABE-2138-46AF-838C-CE23E35B4A09}" name="OX mdot (kg/s)">
+      <calculatedColumnFormula>7.209/2.205</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{A89FC2E7-A5A5-4B36-A697-D725530FD1AF}" name="OX Tank Pressure (psi)"/>
+    <tableColumn id="9" xr3:uid="{A64DC4F4-A184-4D0B-8E07-BC4209542B83}" name="OX Press Gas"/>
+    <tableColumn id="10" xr3:uid="{3F2BA43E-8364-4D07-8B5F-8A76FB3F8E6E}" name="OX Source Pressure (psi)"/>
+    <tableColumn id="11" xr3:uid="{375A1EBD-2658-41BB-A916-BF3F722D5A95}" name="OX Source Temperature (K)"/>
+    <tableColumn id="5" xr3:uid="{6F1CAFC6-53BA-4008-ABF6-539843B7C312}" name="Fuel"/>
+    <tableColumn id="4" xr3:uid="{1C2FF809-5FFB-459A-B5D7-42BEF4C04AA2}" name="FU mdot (kg/s)">
+      <calculatedColumnFormula>4.29/2.205</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="16" xr3:uid="{153B6794-733E-497F-AA6F-C8DC855F4143}" name="FU Tank Pressure (psi)"/>
+    <tableColumn id="12" xr3:uid="{516A76CC-8D45-4E24-9F7F-142004617BC1}" name="FU Press Gas"/>
+    <tableColumn id="13" xr3:uid="{5BB4A00F-DA34-4B22-A583-3BCE9D881BFE}" name="FU Source Pressure (psi)" dataDxfId="0"/>
+    <tableColumn id="14" xr3:uid="{303A5C50-F899-4E2C-B94B-A2D11BB69A68}" name="FU Source Temperature (K)"/>
+    <tableColumn id="8" xr3:uid="{7659E010-E8AA-4FAC-86E8-2222973BDFFE}" name="Fill Pressure (used for prop density) (psi)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -513,149 +648,437 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7708522A-A771-4A2F-B747-04EC8410C62A}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="41" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="28" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="27.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="36.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="51.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="36" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="28" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.5703125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+      <c r="H1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J1" t="s">
+        <v>18</v>
+      </c>
+      <c r="K1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L1" t="s">
+        <v>1</v>
+      </c>
+      <c r="M1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" t="s">
+      <c r="N1" t="s">
+        <v>16</v>
+      </c>
+      <c r="O1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P1" t="s">
+        <v>21</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>22</v>
+      </c>
+      <c r="R1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="1">
         <v>1</v>
       </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" t="s">
-        <v>2</v>
-      </c>
-      <c r="J1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
+      <c r="D2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="1">
+        <v>3.4</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="1">
+        <f>7.209/2.205</f>
+        <v>3.2693877551020405</v>
+      </c>
+      <c r="H2" s="1">
+        <v>1055</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="1">
+        <v>1842</v>
+      </c>
+      <c r="K2" s="1">
+        <v>288.70600000000002</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M2" s="1">
+        <f>4.29/2.205</f>
+        <v>1.9455782312925169</v>
+      </c>
+      <c r="N2" s="1">
+        <v>1055</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="P2" s="1">
+        <v>1842</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>288.70600000000002</v>
+      </c>
+      <c r="R2" s="1">
+        <v>14.7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{088C9C01-56F8-4798-8850-4C6BA490C79B}">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" t="s">
-        <v>22</v>
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A2" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
+      <c r="A3" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="6">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <f>0.5-0.089*2</f>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>18</v>
+      <c r="A4" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="7"/>
+      <c r="C4">
+        <f t="shared" ref="C4:C19" si="0">0.5-0.089*2</f>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D4" s="7">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>19</v>
-      </c>
+      <c r="A5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="6">
+        <v>3</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
+      <c r="A6" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="7"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>17</v>
+      <c r="A7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="7"/>
+      <c r="C7" s="9">
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D7" s="7">
+        <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
+      <c r="A8" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="7">
+        <v>3</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D8" s="7"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="7"/>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D9" s="7">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="7">
+        <v>6</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D10" s="7"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D11" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="C12">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D12" s="7"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="9">
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D14" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" s="7">
+        <v>8</v>
+      </c>
+      <c r="C15">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D15" s="7"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" s="7"/>
+      <c r="C16">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D16" s="7">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="7">
+        <v>6</v>
+      </c>
+      <c r="C17">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D17" s="7"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B18" s="7"/>
+      <c r="C18">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D18" s="7">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="7">
+        <v>0.5</v>
+      </c>
+      <c r="C19">
+        <f t="shared" si="0"/>
+        <v>0.32200000000000001</v>
+      </c>
+      <c r="D19" s="7"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Many updates over time
</commit_message>
<xml_diff>
--- a/Pressurization_System/Press System Test Cases.xlsx
+++ b/Pressurization_System/Press System Test Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://purdue0-my.sharepoint.com/personal/tucke193_purdue_edu/Documents/PSP/Test Stand/PSPL_Test_Stand/Pressurization_System/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="349" documentId="8_{3BA32EE1-FD8D-41E0-A269-E64256623536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2F25E5AB-9888-4037-ACA2-3C0026F22B04}"/>
+  <xr:revisionPtr revIDLastSave="373" documentId="8_{3BA32EE1-FD8D-41E0-A269-E64256623536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2466051F-BE0A-4E2A-859E-6A8628D27240}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{C0027B85-AECA-41BE-812F-CA93B39DA64E}"/>
+    <workbookView minimized="1" xWindow="3510" yWindow="3510" windowWidth="28800" windowHeight="15030" activeTab="1" xr2:uid="{C0027B85-AECA-41BE-812F-CA93B39DA64E}"/>
   </bookViews>
   <sheets>
     <sheet name="Initial Conditions" sheetId="1" r:id="rId1"/>
@@ -274,7 +274,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -294,10 +294,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -841,8 +837,8 @@
         <v>10</v>
       </c>
       <c r="C3">
-        <f>0.5-0.089*2</f>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D3" s="6"/>
     </row>
@@ -852,7 +848,7 @@
       </c>
       <c r="B4" s="7"/>
       <c r="C4">
-        <f t="shared" ref="C4:C19" si="0">0.5-0.089*2</f>
+        <f t="shared" ref="C4:C18" si="0">0.5-0.089*2</f>
         <v>0.32200000000000001</v>
       </c>
       <c r="D4" s="7">
@@ -867,8 +863,8 @@
         <v>3</v>
       </c>
       <c r="C5">
-        <f t="shared" si="0"/>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D5" s="6"/>
     </row>
@@ -900,8 +896,8 @@
         <v>3</v>
       </c>
       <c r="C8">
-        <f t="shared" si="0"/>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D8" s="7"/>
     </row>
@@ -926,8 +922,8 @@
         <v>6</v>
       </c>
       <c r="C10">
-        <f t="shared" si="0"/>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D10" s="7"/>
     </row>
@@ -952,8 +948,8 @@
         <v>0.5</v>
       </c>
       <c r="C12">
-        <f t="shared" si="0"/>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D12" s="7"/>
     </row>
@@ -985,8 +981,8 @@
         <v>8</v>
       </c>
       <c r="C15">
-        <f t="shared" si="0"/>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D15" s="7"/>
     </row>
@@ -1011,8 +1007,8 @@
         <v>6</v>
       </c>
       <c r="C17">
-        <f t="shared" si="0"/>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D17" s="7"/>
     </row>
@@ -1037,8 +1033,8 @@
         <v>0.5</v>
       </c>
       <c r="C19">
-        <f t="shared" si="0"/>
-        <v>0.32200000000000001</v>
+        <f>0.75-0.12*2</f>
+        <v>0.51</v>
       </c>
       <c r="D19" s="7"/>
     </row>

</xml_diff>